<commit_message>
Update JPM data - 2026-09-06 16:10:47
</commit_message>
<xml_diff>
--- a/data/JPM_data.xlsx
+++ b/data/JPM_data.xlsx
@@ -3897,7 +3897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4018,25 +4018,45 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>book_value</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>price_to_book</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>earnings_growth</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>shares_outstanding</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -4096,7 +4116,7 @@
         <v>0.975</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.66</v>
+        <v>1.67</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -4124,29 +4144,41 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" t="n">
+        <v>133.007</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>2.6963995</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0.469</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>2658186195</v>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Financial Services</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Banks - Diversified</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>https://www.jpmorganchase.com</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>JPMorgan Chase &amp; Co. operates as a bank and financial holding company in the United States, rest of North America, Europe, the Middle East, Africa, the Asia Pacific, Latin America, and the Caribbean. It operates in three segments: Consumer &amp; Community Banking, Commercial &amp; Investment Bank, and Asset &amp; Wealth Management. The company offers deposit, investment and lending products, and cash management; mortgage origination and servicing activities; residential mortgages and home equity loans; and credit cards, payment solutions, travel services, merchant offers, lifestyle benefits, auto loans, and leases to consumers and small businesses through bank branches, ATMs, and digital and telephone banking. It also provides investment banking, market-making, financing, custody, and securities products and services; corporate strategy and structure advisory, equity and debt market capital-raising, and loan origination and syndication services; cash and derivative instruments, risk management solutions, prime brokerage, clearing, and research; and fund services, liquidity and trading services, and data solutions products for large corporations, financial institutions, merchants, start-ups, small and midsized companies, local governments, municipalities, nonprofits, and commercial real estate clients. In addition, the company offers multi-asset investment management solutions in equities, fixed income, alternatives, and money market funds to institutional clients and retail investors; retirement products and services, estate planning, lending, deposits, and investment management products to high-net-worth clients; and financial transaction processing. JPMorgan Chase &amp; Co. was founded in 1799 and is headquartered in New York, New York.</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>2026-09-06 05:41:59</t>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>2026-09-06 16:10:02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update JPM data - 2026-09-06 17:00:22
</commit_message>
<xml_diff>
--- a/data/JPM_data.xlsx
+++ b/data/JPM_data.xlsx
@@ -4118,15 +4118,11 @@
       <c r="Q2" t="n">
         <v>1.67</v>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="R2" t="n">
+        <v>0.34921002</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.5039400000000001</v>
       </c>
       <c r="T2" t="n">
         <v>0.17789</v>
@@ -4178,7 +4174,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>2026-09-06 16:49:07</t>
+          <t>2026-09-06 16:59:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update JPM data - 2026-09-06 22:21:27
</commit_message>
<xml_diff>
--- a/data/JPM_data.xlsx
+++ b/data/JPM_data.xlsx
@@ -3897,7 +3897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4038,25 +4038,40 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>total_revenue</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>enterprise_value</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>ebitda</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -4152,29 +4167,40 @@
       <c r="AA2" t="n">
         <v>2658186195</v>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB2" t="n">
+        <v>186328006656</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>791259906048</v>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Financial Services</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>Banks - Diversified</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>https://www.jpmorganchase.com</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>JPMorgan Chase &amp; Co. operates as a bank and financial holding company in the United States, rest of North America, Europe, the Middle East, Africa, the Asia Pacific, Latin America, and the Caribbean. It operates in three segments: Consumer &amp; Community Banking, Commercial &amp; Investment Bank, and Asset &amp; Wealth Management. The company offers deposit, investment and lending products, and cash management; mortgage origination and servicing activities; residential mortgages and home equity loans; and credit cards, payment solutions, travel services, merchant offers, lifestyle benefits, auto loans, and leases to consumers and small businesses through bank branches, ATMs, and digital and telephone banking. It also provides investment banking, market-making, financing, custody, and securities products and services; corporate strategy and structure advisory, equity and debt market capital-raising, and loan origination and syndication services; cash and derivative instruments, risk management solutions, prime brokerage, clearing, and research; and fund services, liquidity and trading services, and data solutions products for large corporations, financial institutions, merchants, start-ups, small and midsized companies, local governments, municipalities, nonprofits, and commercial real estate clients. In addition, the company offers multi-asset investment management solutions in equities, fixed income, alternatives, and money market funds to institutional clients and retail investors; retirement products and services, estate planning, lending, deposits, and investment management products to high-net-worth clients; and financial transaction processing. JPMorgan Chase &amp; Co. was founded in 1799 and is headquartered in New York, New York.</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>2026-09-06 16:59:37</t>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>2026-09-06 22:20:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update JPM data - 2026-09-08 08:53:13
</commit_message>
<xml_diff>
--- a/data/JPM_data.xlsx
+++ b/data/JPM_data.xlsx
@@ -472,16 +472,16 @@
         <v>45905</v>
       </c>
       <c r="B2" t="n">
-        <v>297.9499798501053</v>
+        <v>297.9500113286781</v>
       </c>
       <c r="C2" t="n">
-        <v>299.4218223620716</v>
+        <v>299.4218539961453</v>
       </c>
       <c r="D2" t="n">
-        <v>288.7853107356273</v>
+        <v>288.7853412459479</v>
       </c>
       <c r="E2" t="n">
-        <v>288.85400390625</v>
+        <v>288.8540344238281</v>
       </c>
       <c r="F2" t="n">
         <v>9837700</v>
@@ -498,16 +498,16 @@
         <v>45908</v>
       </c>
       <c r="B3" t="n">
-        <v>289.3544334283243</v>
+        <v>289.3544641521949</v>
       </c>
       <c r="C3" t="n">
-        <v>290.894939131519</v>
+        <v>290.8949700189617</v>
       </c>
       <c r="D3" t="n">
-        <v>285.9691837491296</v>
+        <v>285.9692141135519</v>
       </c>
       <c r="E3" t="n">
-        <v>287.4115905761719</v>
+        <v>287.41162109375</v>
       </c>
       <c r="F3" t="n">
         <v>8188500</v>
@@ -524,16 +524,16 @@
         <v>45909</v>
       </c>
       <c r="B4" t="n">
-        <v>287.1074615709347</v>
+        <v>287.1074315912692</v>
       </c>
       <c r="C4" t="n">
-        <v>293.3873179050423</v>
+        <v>293.3872872696363</v>
       </c>
       <c r="D4" t="n">
-        <v>286.8228969249006</v>
+        <v>286.8228669749493</v>
       </c>
       <c r="E4" t="n">
-        <v>292.2589111328125</v>
+        <v>292.2588806152344</v>
       </c>
       <c r="F4" t="n">
         <v>7848200</v>
@@ -576,16 +576,16 @@
         <v>45911</v>
       </c>
       <c r="B6" t="n">
-        <v>295.5852436958139</v>
+        <v>295.5852136096933</v>
       </c>
       <c r="C6" t="n">
-        <v>299.9909797241969</v>
+        <v>299.9909491896388</v>
       </c>
       <c r="D6" t="n">
-        <v>295.1437088676121</v>
+        <v>295.1436788264331</v>
       </c>
       <c r="E6" t="n">
-        <v>299.8241577148438</v>
+        <v>299.8241271972656</v>
       </c>
       <c r="F6" t="n">
         <v>7942500</v>
@@ -628,16 +628,16 @@
         <v>45915</v>
       </c>
       <c r="B8" t="n">
-        <v>301.4039041511534</v>
+        <v>301.4039344978193</v>
       </c>
       <c r="C8" t="n">
-        <v>304.1317175736464</v>
+        <v>304.1317481949604</v>
       </c>
       <c r="D8" t="n">
-        <v>301.4039041511534</v>
+        <v>301.4039344978193</v>
       </c>
       <c r="E8" t="n">
-        <v>303.1014099121094</v>
+        <v>303.1014404296875</v>
       </c>
       <c r="F8" t="n">
         <v>7122000</v>
@@ -940,16 +940,16 @@
         <v>45931</v>
       </c>
       <c r="B20" t="n">
-        <v>308.0762861336198</v>
+        <v>308.0763169713923</v>
       </c>
       <c r="C20" t="n">
-        <v>308.6846429587351</v>
+        <v>308.6846738574029</v>
       </c>
       <c r="D20" t="n">
-        <v>301.6394301376976</v>
+        <v>301.6394603311547</v>
       </c>
       <c r="E20" t="n">
-        <v>304.8774719238281</v>
+        <v>304.8775024414062</v>
       </c>
       <c r="F20" t="n">
         <v>9235200</v>
@@ -992,16 +992,16 @@
         <v>45933</v>
       </c>
       <c r="B22" t="n">
-        <v>302.718779227698</v>
+        <v>302.7188095956571</v>
       </c>
       <c r="C22" t="n">
-        <v>305.8096426575195</v>
+        <v>305.809673335546</v>
       </c>
       <c r="D22" t="n">
-        <v>302.4243927447969</v>
+        <v>302.4244230832239</v>
       </c>
       <c r="E22" t="n">
-        <v>304.2102355957031</v>
+        <v>304.2102661132812</v>
       </c>
       <c r="F22" t="n">
         <v>6029900</v>
@@ -1018,16 +1018,16 @@
         <v>45936</v>
       </c>
       <c r="B23" t="n">
-        <v>305.8371341622301</v>
+        <v>305.8371035459471</v>
       </c>
       <c r="C23" t="n">
-        <v>307.3851596699703</v>
+        <v>307.3851288987199</v>
       </c>
       <c r="D23" t="n">
-        <v>300.857851711314</v>
+        <v>300.8578215934895</v>
       </c>
       <c r="E23" t="n">
-        <v>304.8511352539062</v>
+        <v>304.8511047363281</v>
       </c>
       <c r="F23" t="n">
         <v>7214500</v>
@@ -1070,16 +1070,16 @@
         <v>45938</v>
       </c>
       <c r="B25" t="n">
-        <v>303.8946917756213</v>
+        <v>303.894722712774</v>
       </c>
       <c r="C25" t="n">
-        <v>304.4567183318842</v>
+        <v>304.4567493262524</v>
       </c>
       <c r="D25" t="n">
-        <v>299.2999336047902</v>
+        <v>299.2999640741864</v>
       </c>
       <c r="E25" t="n">
-        <v>299.7732238769531</v>
+        <v>299.7732543945312</v>
       </c>
       <c r="F25" t="n">
         <v>6489900</v>
@@ -1148,16 +1148,16 @@
         <v>45943</v>
       </c>
       <c r="B28" t="n">
-        <v>301.3212684867699</v>
+        <v>301.321238204041</v>
       </c>
       <c r="C28" t="n">
-        <v>305.1272097801061</v>
+        <v>305.1271791148808</v>
       </c>
       <c r="D28" t="n">
-        <v>301.1733746705027</v>
+        <v>301.173344402637</v>
       </c>
       <c r="E28" t="n">
-        <v>303.6580810546875</v>
+        <v>303.6580505371094</v>
       </c>
       <c r="F28" t="n">
         <v>10788700</v>
@@ -1200,16 +1200,16 @@
         <v>45945</v>
       </c>
       <c r="B30" t="n">
-        <v>302.1002149225357</v>
+        <v>302.1001843350741</v>
       </c>
       <c r="C30" t="n">
-        <v>307.7499693151439</v>
+        <v>307.7499381556482</v>
       </c>
       <c r="D30" t="n">
-        <v>301.1635039391426</v>
+        <v>301.1634734465224</v>
       </c>
       <c r="E30" t="n">
-        <v>301.4100036621094</v>
+        <v>301.4099731445312</v>
       </c>
       <c r="F30" t="n">
         <v>11354800</v>
@@ -1226,16 +1226,16 @@
         <v>45946</v>
       </c>
       <c r="B31" t="n">
-        <v>301.0747260223031</v>
+        <v>301.0747572360179</v>
       </c>
       <c r="C31" t="n">
-        <v>304.358088638523</v>
+        <v>304.3581201926382</v>
       </c>
       <c r="D31" t="n">
-        <v>292.9106575300408</v>
+        <v>292.9106878973514</v>
       </c>
       <c r="E31" t="n">
-        <v>294.3600769042969</v>
+        <v>294.360107421875</v>
       </c>
       <c r="F31" t="n">
         <v>10549400</v>
@@ -1356,16 +1356,16 @@
         <v>45953</v>
       </c>
       <c r="B36" t="n">
-        <v>290.2583742532713</v>
+        <v>290.2583437522712</v>
       </c>
       <c r="C36" t="n">
-        <v>292.220502524991</v>
+        <v>292.2204718178062</v>
       </c>
       <c r="D36" t="n">
-        <v>288.4145610405075</v>
+        <v>288.4145307332595</v>
       </c>
       <c r="E36" t="n">
-        <v>290.4161376953125</v>
+        <v>290.4161071777344</v>
       </c>
       <c r="F36" t="n">
         <v>5438800</v>
@@ -1382,16 +1382,16 @@
         <v>45954</v>
       </c>
       <c r="B37" t="n">
-        <v>291.9345495322769</v>
+        <v>291.9345194575729</v>
       </c>
       <c r="C37" t="n">
-        <v>298.3632818043669</v>
+        <v>298.3632510673837</v>
       </c>
       <c r="D37" t="n">
-        <v>291.3133954831271</v>
+        <v>291.3133654724136</v>
       </c>
       <c r="E37" t="n">
-        <v>296.2335205078125</v>
+        <v>296.2334899902344</v>
       </c>
       <c r="F37" t="n">
         <v>7228300</v>
@@ -1486,16 +1486,16 @@
         <v>45960</v>
       </c>
       <c r="B41" t="n">
-        <v>301.5086233262724</v>
+        <v>301.5085931686638</v>
       </c>
       <c r="C41" t="n">
-        <v>308.233113206998</v>
+        <v>308.2330823767899</v>
       </c>
       <c r="D41" t="n">
-        <v>300.8282816526182</v>
+        <v>300.828251563059</v>
       </c>
       <c r="E41" t="n">
-        <v>305.1075134277344</v>
+        <v>305.1074829101562</v>
       </c>
       <c r="F41" t="n">
         <v>7514600</v>
@@ -1616,16 +1616,16 @@
         <v>45967</v>
       </c>
       <c r="B46" t="n">
-        <v>306.6357990367445</v>
+        <v>306.6357687557767</v>
       </c>
       <c r="C46" t="n">
-        <v>310.4319009529449</v>
+        <v>310.4318702971036</v>
       </c>
       <c r="D46" t="n">
-        <v>305.9160390722913</v>
+        <v>305.9160088624015</v>
       </c>
       <c r="E46" t="n">
-        <v>309.0317993164062</v>
+        <v>309.0317687988281</v>
       </c>
       <c r="F46" t="n">
         <v>7206100</v>
@@ -1746,16 +1746,16 @@
         <v>45974</v>
       </c>
       <c r="B51" t="n">
-        <v>314.7604311532612</v>
+        <v>314.7604626322791</v>
       </c>
       <c r="C51" t="n">
-        <v>316.1408235578094</v>
+        <v>316.1408551748796</v>
       </c>
       <c r="D51" t="n">
-        <v>304.7722577523736</v>
+        <v>304.7722882324798</v>
       </c>
       <c r="E51" t="n">
-        <v>305.1469421386719</v>
+        <v>305.14697265625</v>
       </c>
       <c r="F51" t="n">
         <v>8973300</v>
@@ -1850,16 +1850,16 @@
         <v>45980</v>
       </c>
       <c r="B55" t="n">
-        <v>295.5432899586994</v>
+        <v>295.5432597963394</v>
       </c>
       <c r="C55" t="n">
-        <v>300.1873662746028</v>
+        <v>300.1873356382808</v>
       </c>
       <c r="D55" t="n">
-        <v>295.0798692888629</v>
+        <v>295.0798391737984</v>
       </c>
       <c r="E55" t="n">
-        <v>299.0238647460938</v>
+        <v>299.0238342285156</v>
       </c>
       <c r="F55" t="n">
         <v>5546600</v>
@@ -1876,16 +1876,16 @@
         <v>45981</v>
       </c>
       <c r="B56" t="n">
-        <v>302.0509050250311</v>
+        <v>302.0508736933244</v>
       </c>
       <c r="C56" t="n">
-        <v>305.5807980031574</v>
+        <v>305.5807663052954</v>
       </c>
       <c r="D56" t="n">
-        <v>293.9854410949062</v>
+        <v>293.9854105998292</v>
       </c>
       <c r="E56" t="n">
-        <v>294.2023620605469</v>
+        <v>294.2023315429688</v>
       </c>
       <c r="F56" t="n">
         <v>7501600</v>
@@ -1902,16 +1902,16 @@
         <v>45982</v>
       </c>
       <c r="B57" t="n">
-        <v>297.0716172552904</v>
+        <v>297.0715864028587</v>
       </c>
       <c r="C57" t="n">
-        <v>297.4561411796575</v>
+        <v>297.456110287291</v>
       </c>
       <c r="D57" t="n">
-        <v>288.7103357437745</v>
+        <v>288.7103057597054</v>
       </c>
       <c r="E57" t="n">
-        <v>293.8473815917969</v>
+        <v>293.8473510742188</v>
       </c>
       <c r="F57" t="n">
         <v>11766800</v>
@@ -1954,16 +1954,16 @@
         <v>45986</v>
       </c>
       <c r="B59" t="n">
-        <v>295.8489209666184</v>
+        <v>295.848951187077</v>
       </c>
       <c r="C59" t="n">
-        <v>300.2366275598507</v>
+        <v>300.236658228506</v>
       </c>
       <c r="D59" t="n">
-        <v>291.4217960873232</v>
+        <v>291.4218258555586</v>
       </c>
       <c r="E59" t="n">
-        <v>298.7576293945312</v>
+        <v>298.7576599121094</v>
       </c>
       <c r="F59" t="n">
         <v>8877200</v>
@@ -2032,16 +2032,16 @@
         <v>45992</v>
       </c>
       <c r="B62" t="n">
-        <v>308.5683618849884</v>
+        <v>308.5683309692949</v>
       </c>
       <c r="C62" t="n">
-        <v>309.6430970545817</v>
+        <v>309.6430660312097</v>
       </c>
       <c r="D62" t="n">
-        <v>304.2201032083801</v>
+        <v>304.2200727283419</v>
       </c>
       <c r="E62" t="n">
-        <v>304.5947875976562</v>
+        <v>304.5947570800781</v>
       </c>
       <c r="F62" t="n">
         <v>7727300</v>
@@ -2110,16 +2110,16 @@
         <v>45995</v>
       </c>
       <c r="B65" t="n">
-        <v>308.8740523757101</v>
+        <v>308.8740221323167</v>
       </c>
       <c r="C65" t="n">
-        <v>314.0308078212495</v>
+        <v>314.0307770729326</v>
       </c>
       <c r="D65" t="n">
-        <v>308.617683010128</v>
+        <v>308.617652791837</v>
       </c>
       <c r="E65" t="n">
-        <v>311.6742858886719</v>
+        <v>311.6742553710938</v>
       </c>
       <c r="F65" t="n">
         <v>9627800</v>
@@ -2136,16 +2136,16 @@
         <v>45996</v>
       </c>
       <c r="B66" t="n">
-        <v>311.2207252653726</v>
+        <v>311.2206946896725</v>
       </c>
       <c r="C66" t="n">
-        <v>314.0209586927274</v>
+        <v>314.0209278419201</v>
       </c>
       <c r="D66" t="n">
-        <v>310.2741446015314</v>
+        <v>310.2741141188276</v>
       </c>
       <c r="E66" t="n">
-        <v>310.6291198730469</v>
+        <v>310.6290893554688</v>
       </c>
       <c r="F66" t="n">
         <v>6518900</v>
@@ -2292,16 +2292,16 @@
         <v>46006</v>
       </c>
       <c r="B72" t="n">
-        <v>315.1153648797306</v>
+        <v>315.115395356304</v>
       </c>
       <c r="C72" t="n">
-        <v>318.3593094805321</v>
+        <v>318.3593402708456</v>
       </c>
       <c r="D72" t="n">
-        <v>313.9321843288561</v>
+        <v>313.9322146909975</v>
       </c>
       <c r="E72" t="n">
-        <v>315.5393371582031</v>
+        <v>315.5393676757812</v>
       </c>
       <c r="F72" t="n">
         <v>10864100</v>
@@ -2344,16 +2344,16 @@
         <v>46008</v>
       </c>
       <c r="B74" t="n">
-        <v>313.9716244610726</v>
+        <v>313.971593609235</v>
       </c>
       <c r="C74" t="n">
-        <v>314.8984658400699</v>
+        <v>314.8984348971578</v>
       </c>
       <c r="D74" t="n">
-        <v>310.2544194174254</v>
+        <v>310.254388930852</v>
       </c>
       <c r="E74" t="n">
-        <v>310.5699462890625</v>
+        <v>310.5699157714844</v>
       </c>
       <c r="F74" t="n">
         <v>8718700</v>
@@ -2370,16 +2370,16 @@
         <v>46009</v>
       </c>
       <c r="B75" t="n">
-        <v>311.5756418636432</v>
+        <v>311.575672673722</v>
       </c>
       <c r="C75" t="n">
-        <v>313.2518519730792</v>
+        <v>313.2518829489097</v>
       </c>
       <c r="D75" t="n">
-        <v>307.8485673512913</v>
+        <v>307.8485977928193</v>
       </c>
       <c r="E75" t="n">
-        <v>308.6176452636719</v>
+        <v>308.61767578125</v>
       </c>
       <c r="F75" t="n">
         <v>11444900</v>
@@ -2422,16 +2422,16 @@
         <v>46013</v>
       </c>
       <c r="B77" t="n">
-        <v>313.064515200958</v>
+        <v>313.0644852104395</v>
       </c>
       <c r="C77" t="n">
-        <v>318.7044300194866</v>
+        <v>318.7043994886834</v>
       </c>
       <c r="D77" t="n">
-        <v>313.064515200958</v>
+        <v>313.0644852104395</v>
       </c>
       <c r="E77" t="n">
-        <v>318.5663757324219</v>
+        <v>318.5663452148438</v>
       </c>
       <c r="F77" t="n">
         <v>8354600</v>
@@ -2500,16 +2500,16 @@
         <v>46017</v>
       </c>
       <c r="B80" t="n">
-        <v>324.5020893383847</v>
+        <v>324.502058709128</v>
       </c>
       <c r="C80" t="n">
-        <v>326.22758744424</v>
+        <v>326.2275566521161</v>
       </c>
       <c r="D80" t="n">
-        <v>321.9680949886989</v>
+        <v>321.9680645986219</v>
       </c>
       <c r="E80" t="n">
-        <v>323.3189086914062</v>
+        <v>323.3188781738281</v>
       </c>
       <c r="F80" t="n">
         <v>4158300</v>
@@ -2630,16 +2630,16 @@
         <v>46027</v>
       </c>
       <c r="B85" t="n">
-        <v>320.942628937084</v>
+        <v>320.9426586744551</v>
       </c>
       <c r="C85" t="n">
-        <v>332.5281155423397</v>
+        <v>332.5281463531796</v>
       </c>
       <c r="D85" t="n">
-        <v>320.636971697701</v>
+        <v>320.637001406751</v>
       </c>
       <c r="E85" t="n">
-        <v>329.3630676269531</v>
+        <v>329.3630981445312</v>
       </c>
       <c r="F85" t="n">
         <v>10752600</v>
@@ -2682,16 +2682,16 @@
         <v>46029</v>
       </c>
       <c r="B87" t="n">
-        <v>327.9764659913386</v>
+        <v>327.9764350864437</v>
       </c>
       <c r="C87" t="n">
-        <v>328.9767963949314</v>
+        <v>328.9767653957764</v>
       </c>
       <c r="D87" t="n">
-        <v>321.4989374679619</v>
+        <v>321.4989071734381</v>
       </c>
       <c r="E87" t="n">
-        <v>323.8660888671875</v>
+        <v>323.8660583496094</v>
       </c>
       <c r="F87" t="n">
         <v>9815200</v>
@@ -2760,16 +2760,16 @@
         <v>46034</v>
       </c>
       <c r="B90" t="n">
-        <v>318.8049029297019</v>
+        <v>318.8049332018166</v>
       </c>
       <c r="C90" t="n">
-        <v>322.9053354478686</v>
+        <v>322.9053661093398</v>
       </c>
       <c r="D90" t="n">
-        <v>318.1611187929736</v>
+        <v>318.1611490039577</v>
       </c>
       <c r="E90" t="n">
-        <v>321.3899536132812</v>
+        <v>321.3899841308594</v>
       </c>
       <c r="F90" t="n">
         <v>12805100</v>
@@ -2786,16 +2786,16 @@
         <v>46035</v>
       </c>
       <c r="B91" t="n">
-        <v>321.2017547389941</v>
+        <v>321.2017865718998</v>
       </c>
       <c r="C91" t="n">
-        <v>323.7372950994605</v>
+        <v>323.7373271836527</v>
       </c>
       <c r="D91" t="n">
-        <v>307.6029450408882</v>
+        <v>307.6029755260753</v>
       </c>
       <c r="E91" t="n">
-        <v>307.9297790527344</v>
+        <v>307.9298095703125</v>
       </c>
       <c r="F91" t="n">
         <v>19371200</v>
@@ -2968,16 +2968,16 @@
         <v>46045</v>
       </c>
       <c r="B98" t="n">
-        <v>299.1148112655088</v>
+        <v>299.1148422218051</v>
       </c>
       <c r="C98" t="n">
-        <v>299.4812715954647</v>
+        <v>299.4813025896872</v>
       </c>
       <c r="D98" t="n">
-        <v>293.6772702297321</v>
+        <v>293.6773006232809</v>
       </c>
       <c r="E98" t="n">
-        <v>294.8757019042969</v>
+        <v>294.875732421875</v>
       </c>
       <c r="F98" t="n">
         <v>11107900</v>
@@ -2994,16 +2994,16 @@
         <v>46048</v>
       </c>
       <c r="B99" t="n">
-        <v>294.9648486176391</v>
+        <v>294.9648788077786</v>
       </c>
       <c r="C99" t="n">
-        <v>298.8969221500132</v>
+        <v>298.8969527426069</v>
       </c>
       <c r="D99" t="n">
-        <v>294.6083024116733</v>
+        <v>294.6083325653198</v>
       </c>
       <c r="E99" t="n">
-        <v>298.1640014648438</v>
+        <v>298.1640319824219</v>
       </c>
       <c r="F99" t="n">
         <v>11752700</v>
@@ -3124,16 +3124,16 @@
         <v>46055</v>
       </c>
       <c r="B104" t="n">
-        <v>301.5513314360023</v>
+        <v>301.5513012828864</v>
       </c>
       <c r="C104" t="n">
-        <v>306.3450888451811</v>
+        <v>306.3450582127215</v>
       </c>
       <c r="D104" t="n">
-        <v>298.4908553932551</v>
+        <v>298.4908255461663</v>
       </c>
       <c r="E104" t="n">
-        <v>305.1961975097656</v>
+        <v>305.1961669921875</v>
       </c>
       <c r="F104" t="n">
         <v>9839400</v>
@@ -3176,16 +3176,16 @@
         <v>46057</v>
       </c>
       <c r="B106" t="n">
-        <v>311.4062598905275</v>
+        <v>311.4062901330092</v>
       </c>
       <c r="C106" t="n">
-        <v>316.2594412620415</v>
+        <v>316.2594719758441</v>
       </c>
       <c r="D106" t="n">
-        <v>311.4062598905275</v>
+        <v>311.4062901330092</v>
       </c>
       <c r="E106" t="n">
-        <v>314.2389221191406</v>
+        <v>314.2389526367188</v>
       </c>
       <c r="F106" t="n">
         <v>9848800</v>
@@ -3306,16 +3306,16 @@
         <v>46064</v>
       </c>
       <c r="B111" t="n">
-        <v>320.1519144431551</v>
+        <v>320.1518827061323</v>
       </c>
       <c r="C111" t="n">
-        <v>322.1724337503843</v>
+        <v>322.1724018130651</v>
       </c>
       <c r="D111" t="n">
-        <v>305.7805563960757</v>
+        <v>305.7805260837019</v>
       </c>
       <c r="E111" t="n">
-        <v>307.8505859375</v>
+        <v>307.8505554199219</v>
       </c>
       <c r="F111" t="n">
         <v>8703500</v>
@@ -3332,16 +3332,16 @@
         <v>46065</v>
       </c>
       <c r="B112" t="n">
-        <v>309.2966060076438</v>
+        <v>309.2966374972976</v>
       </c>
       <c r="C112" t="n">
-        <v>310.6238005797982</v>
+        <v>310.6238322045743</v>
       </c>
       <c r="D112" t="n">
-        <v>297.1537232583444</v>
+        <v>297.1537535117247</v>
       </c>
       <c r="E112" t="n">
-        <v>299.7487182617188</v>
+        <v>299.7487487792969</v>
       </c>
       <c r="F112" t="n">
         <v>13443400</v>
@@ -3358,16 +3358,16 @@
         <v>46066</v>
       </c>
       <c r="B113" t="n">
-        <v>295.6680481198895</v>
+        <v>295.6680782309701</v>
       </c>
       <c r="C113" t="n">
-        <v>301.3829431862302</v>
+        <v>301.3829738793206</v>
       </c>
       <c r="D113" t="n">
-        <v>293.6871553220786</v>
+        <v>293.6871852314235</v>
       </c>
       <c r="E113" t="n">
-        <v>299.6595458984375</v>
+        <v>299.6595764160156</v>
       </c>
       <c r="F113" t="n">
         <v>9114500</v>
@@ -3384,16 +3384,16 @@
         <v>46070</v>
       </c>
       <c r="B114" t="n">
-        <v>299.8675549474044</v>
+        <v>299.8675850307636</v>
       </c>
       <c r="C114" t="n">
-        <v>305.2951817518681</v>
+        <v>305.2952123797385</v>
       </c>
       <c r="D114" t="n">
-        <v>299.6100292169066</v>
+        <v>299.6100592744303</v>
       </c>
       <c r="E114" t="n">
-        <v>304.19580078125</v>
+        <v>304.1958312988281</v>
       </c>
       <c r="F114" t="n">
         <v>8896800</v>
@@ -3436,16 +3436,16 @@
         <v>46072</v>
       </c>
       <c r="B116" t="n">
-        <v>304.2354576365961</v>
+        <v>304.2354272061944</v>
       </c>
       <c r="C116" t="n">
-        <v>306.226234501648</v>
+        <v>306.2262038721237</v>
       </c>
       <c r="D116" t="n">
-        <v>302.2050242231491</v>
+        <v>302.2049939958365</v>
       </c>
       <c r="E116" t="n">
-        <v>305.1070251464844</v>
+        <v>305.1069946289062</v>
       </c>
       <c r="F116" t="n">
         <v>6737700</v>
@@ -3488,16 +3488,16 @@
         <v>46076</v>
       </c>
       <c r="B118" t="n">
-        <v>305.8498774375392</v>
+        <v>305.8498457788994</v>
       </c>
       <c r="C118" t="n">
-        <v>308.028871901531</v>
+        <v>308.0288400173425</v>
       </c>
       <c r="D118" t="n">
-        <v>292.2807780649544</v>
+        <v>292.2807478108573</v>
       </c>
       <c r="E118" t="n">
-        <v>294.8262329101562</v>
+        <v>294.8262023925781</v>
       </c>
       <c r="F118" t="n">
         <v>12955400</v>
@@ -3540,16 +3540,16 @@
         <v>46078</v>
       </c>
       <c r="B120" t="n">
-        <v>295.7869207463737</v>
+        <v>295.7869507950724</v>
       </c>
       <c r="C120" t="n">
-        <v>300.7589506810849</v>
+        <v>300.7589812348872</v>
       </c>
       <c r="D120" t="n">
-        <v>294.1724883145502</v>
+        <v>294.1725181992404</v>
       </c>
       <c r="E120" t="n">
-        <v>300.4023742675781</v>
+        <v>300.4024047851562</v>
       </c>
       <c r="F120" t="n">
         <v>8095500</v>
@@ -3800,16 +3800,16 @@
         <v>46092</v>
       </c>
       <c r="B130" t="n">
-        <v>286.0508472723319</v>
+        <v>286.0508166178312</v>
       </c>
       <c r="C130" t="n">
-        <v>287.7049062038017</v>
+        <v>287.7048753720447</v>
       </c>
       <c r="D130" t="n">
-        <v>282.1385715612803</v>
+        <v>282.1385413260368</v>
       </c>
       <c r="E130" t="n">
-        <v>284.7731628417969</v>
+        <v>284.7731323242188</v>
       </c>
       <c r="F130" t="n">
         <v>10205000</v>
@@ -3826,16 +3826,16 @@
         <v>46093</v>
       </c>
       <c r="B131" t="n">
-        <v>280.1279843639117</v>
+        <v>280.1279538528093</v>
       </c>
       <c r="C131" t="n">
-        <v>281.1679713767581</v>
+        <v>281.167940752382</v>
       </c>
       <c r="D131" t="n">
-        <v>276.4336380780354</v>
+        <v>276.4336079693154</v>
       </c>
       <c r="E131" t="n">
-        <v>280.1874389648438</v>
+        <v>280.1874084472656</v>
       </c>
       <c r="F131" t="n">
         <v>13760500</v>
@@ -3930,16 +3930,16 @@
         <v>46099</v>
       </c>
       <c r="B135" t="n">
-        <v>284.0897180113691</v>
+        <v>284.0897484324327</v>
       </c>
       <c r="C135" t="n">
-        <v>286.6450865635814</v>
+        <v>286.6451172582804</v>
       </c>
       <c r="D135" t="n">
-        <v>282.3960631878955</v>
+        <v>282.3960934275981</v>
       </c>
       <c r="E135" t="n">
-        <v>284.9910278320312</v>
+        <v>284.9910583496094</v>
       </c>
       <c r="F135" t="n">
         <v>10057000</v>
@@ -3956,16 +3956,16 @@
         <v>46100</v>
       </c>
       <c r="B136" t="n">
-        <v>284.1392890417467</v>
+        <v>284.1392586396808</v>
       </c>
       <c r="C136" t="n">
-        <v>286.7441681021885</v>
+        <v>286.7441374214082</v>
       </c>
       <c r="D136" t="n">
-        <v>281.900870340191</v>
+        <v>281.9008401776293</v>
       </c>
       <c r="E136" t="n">
-        <v>285.2188720703125</v>
+        <v>285.2188415527344</v>
       </c>
       <c r="F136" t="n">
         <v>9846700</v>
@@ -3982,16 +3982,16 @@
         <v>46101</v>
       </c>
       <c r="B137" t="n">
-        <v>285.3277943529036</v>
+        <v>285.327825032355</v>
       </c>
       <c r="C137" t="n">
-        <v>287.9326733008621</v>
+        <v>287.9327042603992</v>
       </c>
       <c r="D137" t="n">
-        <v>282.5446423017302</v>
+        <v>282.5446726819272</v>
       </c>
       <c r="E137" t="n">
-        <v>283.8223266601562</v>
+        <v>283.8223571777344</v>
       </c>
       <c r="F137" t="n">
         <v>22436500</v>
@@ -4086,16 +4086,16 @@
         <v>46107</v>
       </c>
       <c r="B141" t="n">
-        <v>289.7847899387647</v>
+        <v>289.7848205526045</v>
       </c>
       <c r="C141" t="n">
-        <v>292.1717693530369</v>
+        <v>292.1718002190451</v>
       </c>
       <c r="D141" t="n">
-        <v>287.9524883078727</v>
+        <v>287.9525187281419</v>
       </c>
       <c r="E141" t="n">
-        <v>288.8735961914062</v>
+        <v>288.8736267089844</v>
       </c>
       <c r="F141" t="n">
         <v>8669200</v>
@@ -10154,7 +10154,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>2026-09-07 03:08:22</t>
+          <t>2026-09-08 08:52:13</t>
         </is>
       </c>
     </row>

</xml_diff>